<commit_message>
fix(tool): fix embedded timetable data, enforce 100% mindays weight, verify zero violations
</commit_message>
<xml_diff>
--- a/Bao_Cao_Kiem_Dinh_THCS_TKB_FET.xlsx
+++ b/Bao_Cao_Kiem_Dinh_THCS_TKB_FET.xlsx
@@ -405,7 +405,7 @@
         <v>STT</v>
       </c>
       <c r="B1" t="str">
-        <v>Tên Giáo Viên</v>
+        <v>Họ và Tên Giáo Viên</v>
       </c>
       <c r="C1" t="str">
         <v>Chức Vụ / Ghi Chú</v>
@@ -432,7 +432,7 @@
         <v>Thứ 7</v>
       </c>
       <c r="K1" t="str">
-        <v>Số Ngày NghỈ</v>
+        <v>Số Ngày Nghỉ</v>
       </c>
       <c r="L1" t="str">
         <v>Chi Tiết Ngày Nghỉ</v>
@@ -452,7 +452,7 @@
         <v>14</v>
       </c>
       <c r="E2" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F2" t="str">
         <v>3 tiết</v>
@@ -461,7 +461,7 @@
         <v>2 tiết</v>
       </c>
       <c r="H2" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I2" t="str">
         <v>4 tiết</v>
@@ -493,16 +493,16 @@
         <v>4 tiết</v>
       </c>
       <c r="F3" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G3" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H3" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="I3" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J3" t="str">
         <v>NGHỈ</v>
@@ -528,19 +528,19 @@
         <v>19</v>
       </c>
       <c r="E4" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F4" t="str">
         <v>3 tiết</v>
       </c>
       <c r="G4" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H4" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I4" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J4" t="str">
         <v>NGHỈ</v>
@@ -569,16 +569,16 @@
         <v>2 tiết</v>
       </c>
       <c r="F5" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G5" t="str">
         <v>4 tiết</v>
       </c>
       <c r="H5" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I5" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J5" t="str">
         <v>NGHỈ</v>
@@ -607,10 +607,10 @@
         <v>3 tiết</v>
       </c>
       <c r="F6" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G6" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H6" t="str">
         <v>4 tiết</v>
@@ -642,16 +642,16 @@
         <v>18</v>
       </c>
       <c r="E7" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="F7" t="str">
-        <v>2 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="G7" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="H7" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I7" t="str">
         <v>2 tiết</v>
@@ -660,10 +660,10 @@
         <v>4 tiết</v>
       </c>
       <c r="K7">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L7" t="str">
-        <v/>
+        <v>Thứ 2, Thứ 5</v>
       </c>
     </row>
     <row r="8">
@@ -680,7 +680,7 @@
         <v>14</v>
       </c>
       <c r="E8" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F8" t="str">
         <v>NGHỈ</v>
@@ -692,7 +692,7 @@
         <v>2 tiết</v>
       </c>
       <c r="I8" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J8" t="str">
         <v>3 tiết</v>
@@ -721,25 +721,25 @@
         <v>3 tiết</v>
       </c>
       <c r="F9" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G9" t="str">
         <v>4 tiết</v>
       </c>
       <c r="H9" t="str">
-        <v>NGHỈ</v>
+        <v>3 tiết</v>
       </c>
       <c r="I9" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J9" t="str">
-        <v>7 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K9">
         <v>1</v>
       </c>
       <c r="L9" t="str">
-        <v>Thứ 5</v>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="10">
@@ -756,16 +756,16 @@
         <v>20</v>
       </c>
       <c r="E10" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="F10" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G10" t="str">
         <v>6 tiết</v>
       </c>
       <c r="H10" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="I10" t="str">
         <v>4 tiết</v>
@@ -774,10 +774,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="K10">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L10" t="str">
-        <v>Thứ 7</v>
+        <v>Thứ 2, Thứ 7</v>
       </c>
     </row>
     <row r="11">
@@ -794,22 +794,22 @@
         <v>15</v>
       </c>
       <c r="E11" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F11" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G11" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H11" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I11" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J11" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K11">
         <v>1</v>
@@ -835,19 +835,19 @@
         <v>3 tiết</v>
       </c>
       <c r="F12" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G12" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H12" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I12" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="J12" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K12">
         <v>1</v>
@@ -870,16 +870,16 @@
         <v>13</v>
       </c>
       <c r="E13" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F13" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G13" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H13" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I13" t="str">
         <v>3 tiết</v>
@@ -914,22 +914,22 @@
         <v>2 tiết</v>
       </c>
       <c r="G14" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H14" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I14" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J14" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K14">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L14" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="15">
@@ -946,28 +946,28 @@
         <v>16</v>
       </c>
       <c r="E15" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F15" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G15" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H15" t="str">
-        <v>5 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I15" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J15" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K15">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="16">
@@ -984,7 +984,7 @@
         <v>14</v>
       </c>
       <c r="E16" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F16" t="str">
         <v>NGHỈ</v>
@@ -993,13 +993,13 @@
         <v>2 tiết</v>
       </c>
       <c r="H16" t="str">
-        <v>5 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I16" t="str">
         <v>2 tiết</v>
       </c>
       <c r="J16" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K16">
         <v>1</v>
@@ -1022,7 +1022,7 @@
         <v>15</v>
       </c>
       <c r="E17" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F17" t="str">
         <v>4 tiết</v>
@@ -1031,7 +1031,7 @@
         <v>3 tiết</v>
       </c>
       <c r="H17" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I17" t="str">
         <v>3 tiết</v>
@@ -1060,28 +1060,28 @@
         <v>15</v>
       </c>
       <c r="E18" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F18" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G18" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H18" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I18" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="J18" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K18">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L18" t="str">
-        <v/>
+        <v>Thứ 6</v>
       </c>
     </row>
     <row r="19">
@@ -1098,19 +1098,19 @@
         <v>17</v>
       </c>
       <c r="E19" t="str">
-        <v>5 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F19" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G19" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H19" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I19" t="str">
-        <v>4 tiết</v>
+        <v>7 tiết</v>
       </c>
       <c r="J19" t="str">
         <v>NGHỈ</v>
@@ -1174,22 +1174,22 @@
         <v>15</v>
       </c>
       <c r="E21" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F21" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G21" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H21" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I21" t="str">
         <v>3 tiết</v>
       </c>
       <c r="J21" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K21">
         <v>1</v>
@@ -1212,16 +1212,16 @@
         <v>12</v>
       </c>
       <c r="E22" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="F22" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G22" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H22" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I22" t="str">
         <v>2 tiết</v>
@@ -1230,10 +1230,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="K22">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L22" t="str">
-        <v>Thứ 7</v>
+        <v>Thứ 2, Thứ 7</v>
       </c>
     </row>
     <row r="23">
@@ -1253,7 +1253,7 @@
         <v>1 tiết</v>
       </c>
       <c r="F23" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G23" t="str">
         <v>5 tiết</v>
@@ -1262,7 +1262,7 @@
         <v>NGHỈ</v>
       </c>
       <c r="I23" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J23" t="str">
         <v>3 tiết</v>
@@ -1291,25 +1291,25 @@
         <v>4 tiết</v>
       </c>
       <c r="F24" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G24" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H24" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I24" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J24" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K24">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L24" t="str">
-        <v/>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="25">
@@ -1329,25 +1329,25 @@
         <v>3 tiết</v>
       </c>
       <c r="F25" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G25" t="str">
-        <v>2 tiết</v>
+        <v>7 tiết</v>
       </c>
       <c r="H25" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I25" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J25" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L25" t="str">
-        <v>Thứ 7</v>
+        <v>Thứ 3, Thứ 7</v>
       </c>
     </row>
     <row r="26">
@@ -1373,10 +1373,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="H26" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I26" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J26" t="str">
         <v>4 tiết</v>
@@ -1402,28 +1402,28 @@
         <v>15</v>
       </c>
       <c r="E27" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F27" t="str">
         <v>3 tiết</v>
       </c>
       <c r="G27" t="str">
-        <v>NGHỈ</v>
+        <v>1 tiết</v>
       </c>
       <c r="H27" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I27" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J27" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K27">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L27" t="str">
-        <v>Thứ 4</v>
+        <v/>
       </c>
     </row>
     <row r="28">
@@ -1443,10 +1443,10 @@
         <v>3 tiết</v>
       </c>
       <c r="F28" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G28" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H28" t="str">
         <v>2 tiết</v>
@@ -1478,28 +1478,28 @@
         <v>16</v>
       </c>
       <c r="E29" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F29" t="str">
-        <v>2 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="G29" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H29" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I29" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J29" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K29">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L29" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="30">
@@ -1516,19 +1516,19 @@
         <v>15</v>
       </c>
       <c r="E30" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F30" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="G30" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H30" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I30" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J30" t="str">
         <v>2 tiết</v>
@@ -1554,19 +1554,19 @@
         <v>11</v>
       </c>
       <c r="E31" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F31" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G31" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H31" t="str">
         <v>2 tiết</v>
       </c>
       <c r="I31" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J31" t="str">
         <v>NGHỈ</v>
@@ -1592,28 +1592,28 @@
         <v>15</v>
       </c>
       <c r="E32" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F32" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G32" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H32" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I32" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="J32" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K32">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L32" t="str">
-        <v/>
+        <v>Thứ 6</v>
       </c>
     </row>
     <row r="33">
@@ -1630,13 +1630,13 @@
         <v>20</v>
       </c>
       <c r="E33" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F33" t="str">
         <v>4 tiết</v>
       </c>
       <c r="G33" t="str">
-        <v>5 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="H33" t="str">
         <v>4 tiết</v>
@@ -1668,10 +1668,10 @@
         <v>12</v>
       </c>
       <c r="E34" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="F34" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G34" t="str">
         <v>4 tiết</v>
@@ -1686,10 +1686,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="K34">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L34" t="str">
-        <v>Thứ 2, Thứ 7</v>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="35">
@@ -1709,19 +1709,19 @@
         <v>2 tiết</v>
       </c>
       <c r="F35" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G35" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H35" t="str">
-        <v>8 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I35" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J35" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K35">
         <v>1</v>
@@ -1744,28 +1744,28 @@
         <v>17</v>
       </c>
       <c r="E36" t="str">
-        <v>6 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F36" t="str">
-        <v>NGHỈ</v>
+        <v>4 tiết</v>
       </c>
       <c r="G36" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H36" t="str">
-        <v>6 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I36" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="J36" t="str">
-        <v>2 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="K36">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L36" t="str">
-        <v>Thứ 3, Thứ 6</v>
+        <v>Thứ 6</v>
       </c>
     </row>
     <row r="37">
@@ -1785,19 +1785,19 @@
         <v>2 tiết</v>
       </c>
       <c r="F37" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G37" t="str">
         <v>4 tiết</v>
       </c>
       <c r="H37" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I37" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J37" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K37">
         <v>0</v>
@@ -1858,22 +1858,22 @@
         <v>18</v>
       </c>
       <c r="E39" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F39" t="str">
+        <v>2 tiết</v>
+      </c>
+      <c r="G39" t="str">
+        <v>1 tiết</v>
+      </c>
+      <c r="H39" t="str">
+        <v>4 tiết</v>
+      </c>
+      <c r="I39" t="str">
+        <v>2 tiết</v>
+      </c>
+      <c r="J39" t="str">
         <v>5 tiết</v>
-      </c>
-      <c r="G39" t="str">
-        <v>3 tiết</v>
-      </c>
-      <c r="H39" t="str">
-        <v>2 tiết</v>
-      </c>
-      <c r="I39" t="str">
-        <v>2 tiết</v>
-      </c>
-      <c r="J39" t="str">
-        <v>4 tiết</v>
       </c>
       <c r="K39">
         <v>0</v>
@@ -1896,28 +1896,28 @@
         <v>14</v>
       </c>
       <c r="E40" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F40" t="str">
-        <v>NGHỈ</v>
+        <v>1 tiết</v>
       </c>
       <c r="G40" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H40" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I40" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J40" t="str">
         <v>4 tiết</v>
       </c>
       <c r="K40">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L40" t="str">
-        <v>Thứ 3</v>
+        <v/>
       </c>
     </row>
     <row r="41">
@@ -1934,28 +1934,28 @@
         <v>16</v>
       </c>
       <c r="E41" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F41" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G41" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H41" t="str">
         <v>3 tiết</v>
       </c>
       <c r="I41" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J41" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K41">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L41" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="42">
@@ -1975,13 +1975,13 @@
         <v>2 tiết</v>
       </c>
       <c r="F42" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G42" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H42" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I42" t="str">
         <v>4 tiết</v>
@@ -2013,25 +2013,25 @@
         <v>2 tiết</v>
       </c>
       <c r="F43" t="str">
+        <v>4 tiết</v>
+      </c>
+      <c r="G43" t="str">
         <v>5 tiết</v>
       </c>
-      <c r="G43" t="str">
-        <v>2 tiết</v>
-      </c>
       <c r="H43" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I43" t="str">
-        <v>5 tiết</v>
+        <v>7 tiết</v>
       </c>
       <c r="J43" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K43">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L43" t="str">
-        <v/>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="44">
@@ -2051,10 +2051,10 @@
         <v>3 tiết</v>
       </c>
       <c r="F44" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G44" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="H44" t="str">
         <v>2 tiết</v>
@@ -2066,10 +2066,10 @@
         <v>3 tiết</v>
       </c>
       <c r="K44">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L44" t="str">
-        <v/>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="45">
@@ -2089,25 +2089,25 @@
         <v>4 tiết</v>
       </c>
       <c r="F45" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G45" t="str">
-        <v>NGHỈ</v>
+        <v>5 tiết</v>
       </c>
       <c r="H45" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I45" t="str">
-        <v>5 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J45" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K45">
         <v>1</v>
       </c>
       <c r="L45" t="str">
-        <v>Thứ 4</v>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="46">
@@ -2124,22 +2124,22 @@
         <v>21</v>
       </c>
       <c r="E46" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F46" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G46" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H46" t="str">
-        <v>5 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="I46" t="str">
         <v>6 tiết</v>
       </c>
       <c r="J46" t="str">
-        <v>4 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="K46">
         <v>0</v>
@@ -2162,28 +2162,28 @@
         <v>13</v>
       </c>
       <c r="E47" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F47" t="str">
-        <v>3 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G47" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H47" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I47" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J47" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K47">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L47" t="str">
-        <v/>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="48">
@@ -2200,16 +2200,16 @@
         <v>20</v>
       </c>
       <c r="E48" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F48" t="str">
+        <v>4 tiết</v>
+      </c>
+      <c r="G48" t="str">
         <v>5 tiết</v>
       </c>
-      <c r="G48" t="str">
-        <v>4 tiết</v>
-      </c>
       <c r="H48" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I48" t="str">
         <v>2 tiết</v>
@@ -2238,28 +2238,28 @@
         <v>17</v>
       </c>
       <c r="E49" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F49" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G49" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H49" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I49" t="str">
-        <v>6 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J49" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="K49">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L49" t="str">
-        <v/>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="50">
@@ -2276,13 +2276,13 @@
         <v>16</v>
       </c>
       <c r="E50" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F50" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G50" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H50" t="str">
         <v>NGHỈ</v>
@@ -2291,7 +2291,7 @@
         <v>4 tiết</v>
       </c>
       <c r="J50" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K50">
         <v>1</v>
@@ -2314,28 +2314,28 @@
         <v>16</v>
       </c>
       <c r="E51" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F51" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G51" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H51" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I51" t="str">
-        <v>2 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J51" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K51">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L51" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="52">
@@ -2355,10 +2355,10 @@
         <v>2 tiết</v>
       </c>
       <c r="F52" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G52" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H52" t="str">
         <v>2 tiết</v>
@@ -2390,28 +2390,28 @@
         <v>19</v>
       </c>
       <c r="E53" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F53" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="G53" t="str">
         <v>4 tiết</v>
       </c>
       <c r="H53" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I53" t="str">
         <v>4 tiết</v>
       </c>
       <c r="J53" t="str">
-        <v>3 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="K53">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L53" t="str">
-        <v/>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="54">
@@ -2428,7 +2428,7 @@
         <v>16</v>
       </c>
       <c r="E54" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F54" t="str">
         <v>2 tiết</v>
@@ -2437,7 +2437,7 @@
         <v>4 tiết</v>
       </c>
       <c r="H54" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I54" t="str">
         <v>2 tiết</v>
@@ -2466,28 +2466,28 @@
         <v>16</v>
       </c>
       <c r="E55" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F55" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G55" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H55" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I55" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J55" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K55">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L55" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="56">
@@ -2504,10 +2504,10 @@
         <v>12</v>
       </c>
       <c r="E56" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F56" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G56" t="str">
         <v>4 tiết</v>
@@ -2516,7 +2516,7 @@
         <v>2 tiết</v>
       </c>
       <c r="I56" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J56" t="str">
         <v>NGHỈ</v>
@@ -2551,10 +2551,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="H57" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="I57" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="J57" t="str">
         <v>NGHỈ</v>
@@ -2563,7 +2563,7 @@
         <v>4</v>
       </c>
       <c r="L57" t="str">
-        <v>Thứ 2, Thứ 4, Thứ 5, Thứ 7</v>
+        <v>Thứ 2, Thứ 4, Thứ 6, Thứ 7</v>
       </c>
     </row>
     <row r="58">
@@ -2583,25 +2583,25 @@
         <v>3 tiết</v>
       </c>
       <c r="F58" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G58" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H58" t="str">
         <v>2 tiết</v>
       </c>
       <c r="I58" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="J58" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K58">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L58" t="str">
-        <v/>
+        <v>Thứ 6</v>
       </c>
     </row>
     <row r="59">
@@ -2618,28 +2618,28 @@
         <v>15</v>
       </c>
       <c r="E59" t="str">
-        <v>6 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F59" t="str">
         <v>1 tiết</v>
       </c>
       <c r="G59" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H59" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I59" t="str">
         <v>1 tiết</v>
       </c>
       <c r="J59" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="K59">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L59" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="60">
@@ -2656,28 +2656,28 @@
         <v>14</v>
       </c>
       <c r="E60" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F60" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G60" t="str">
         <v>1 tiết</v>
       </c>
       <c r="H60" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I60" t="str">
         <v>1 tiết</v>
       </c>
       <c r="J60" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K60">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L60" t="str">
-        <v/>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="61">
@@ -2694,28 +2694,28 @@
         <v>15</v>
       </c>
       <c r="E61" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F61" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G61" t="str">
-        <v>3 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H61" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I61" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J61" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K61">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L61" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="62">
@@ -2732,28 +2732,28 @@
         <v>18</v>
       </c>
       <c r="E62" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="F62" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G62" t="str">
-        <v>2 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="H62" t="str">
-        <v>2 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="I62" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J62" t="str">
-        <v>6 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="K62">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L62" t="str">
-        <v/>
+        <v>Thứ 2, Thứ 7</v>
       </c>
     </row>
     <row r="63">
@@ -2770,28 +2770,28 @@
         <v>15</v>
       </c>
       <c r="E63" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F63" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G63" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H63" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I63" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="J63" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K63">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L63" t="str">
-        <v/>
+        <v>Thứ 6</v>
       </c>
     </row>
     <row r="64">
@@ -2808,28 +2808,28 @@
         <v>17</v>
       </c>
       <c r="E64" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F64" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G64" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H64" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I64" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J64" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L64" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="65">
@@ -2884,28 +2884,28 @@
         <v>13</v>
       </c>
       <c r="E66" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F66" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G66" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="H66" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I66" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J66" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L66" t="str">
-        <v>Thứ 4</v>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -2925,16 +2925,16 @@
         <v>1 tiết</v>
       </c>
       <c r="F67" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G67" t="str">
         <v>1 tiết</v>
       </c>
       <c r="H67" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I67" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J67" t="str">
         <v>3 tiết</v>
@@ -3001,25 +3001,25 @@
         <v>3 tiết</v>
       </c>
       <c r="F69" t="str">
-        <v>2 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="G69" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H69" t="str">
         <v>3 tiết</v>
       </c>
       <c r="I69" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J69" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L69" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="70">
@@ -3074,22 +3074,22 @@
         <v>17</v>
       </c>
       <c r="E71" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F71" t="str">
         <v>4 tiết</v>
       </c>
       <c r="G71" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H71" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I71" t="str">
         <v>4 tiết</v>
       </c>
       <c r="J71" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="K71">
         <v>0</v>
@@ -3112,19 +3112,19 @@
         <v>16</v>
       </c>
       <c r="E72" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F72" t="str">
         <v>4 tiết</v>
       </c>
       <c r="G72" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H72" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I72" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J72" t="str">
         <v>NGHỈ</v>
@@ -3150,28 +3150,28 @@
         <v>13</v>
       </c>
       <c r="E73" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F73" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="G73" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H73" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I73" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J73" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K73">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L73" t="str">
-        <v>Thứ 3</v>
+        <v>Thứ 3, Thứ 5</v>
       </c>
     </row>
     <row r="74">
@@ -3191,16 +3191,16 @@
         <v>2 tiết</v>
       </c>
       <c r="F74" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G74" t="str">
-        <v>6 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H74" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I74" t="str">
-        <v>4 tiết</v>
+        <v>8 tiết</v>
       </c>
       <c r="J74" t="str">
         <v>NGHỈ</v>
@@ -3229,13 +3229,13 @@
         <v>3 tiết</v>
       </c>
       <c r="F75" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G75" t="str">
-        <v>NGHỈ</v>
+        <v>5 tiết</v>
       </c>
       <c r="H75" t="str">
-        <v>5 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I75" t="str">
         <v>3 tiết</v>
@@ -3244,10 +3244,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="K75">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L75" t="str">
-        <v>Thứ 4, Thứ 7</v>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="76">
@@ -3264,28 +3264,28 @@
         <v>18</v>
       </c>
       <c r="E76" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F76" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G76" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H76" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I76" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J76" t="str">
-        <v>5 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="K76">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L76" t="str">
-        <v/>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="77">
@@ -3305,7 +3305,7 @@
         <v>2 tiết</v>
       </c>
       <c r="F77" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G77" t="str">
         <v>2 tiết</v>
@@ -3314,7 +3314,7 @@
         <v>1 tiết</v>
       </c>
       <c r="I77" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J77" t="str">
         <v>NGHỈ</v>
@@ -3340,19 +3340,19 @@
         <v>12</v>
       </c>
       <c r="E78" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F78" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G78" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H78" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I78" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J78" t="str">
         <v>NGHỈ</v>
@@ -3378,19 +3378,19 @@
         <v>11</v>
       </c>
       <c r="E79" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F79" t="str">
         <v>1 tiết</v>
       </c>
       <c r="G79" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H79" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I79" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J79" t="str">
         <v>NGHỈ</v>
@@ -3416,7 +3416,7 @@
         <v>19</v>
       </c>
       <c r="E80" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F80" t="str">
         <v>4 tiết</v>
@@ -3428,7 +3428,7 @@
         <v>4 tiết</v>
       </c>
       <c r="I80" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J80" t="str">
         <v>NGHỈ</v>
@@ -3454,19 +3454,19 @@
         <v>14</v>
       </c>
       <c r="E81" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F81" t="str">
         <v>4 tiết</v>
       </c>
       <c r="G81" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="H81" t="str">
         <v>2 tiết</v>
       </c>
       <c r="I81" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="J81" t="str">
         <v>3 tiết</v>
@@ -3475,7 +3475,7 @@
         <v>1</v>
       </c>
       <c r="L81" t="str">
-        <v>Thứ 4</v>
+        <v>Thứ 6</v>
       </c>
     </row>
     <row r="82">
@@ -3495,25 +3495,25 @@
         <v>2 tiết</v>
       </c>
       <c r="F82" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G82" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H82" t="str">
         <v>4 tiết</v>
       </c>
       <c r="I82" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J82" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="K82">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L82" t="str">
-        <v/>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="83">
@@ -3530,19 +3530,19 @@
         <v>14</v>
       </c>
       <c r="E83" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F83" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G83" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H83" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I83" t="str">
-        <v>NGHỈ</v>
+        <v>4 tiết</v>
       </c>
       <c r="J83" t="str">
         <v>3 tiết</v>
@@ -3551,7 +3551,7 @@
         <v>1</v>
       </c>
       <c r="L83" t="str">
-        <v>Thứ 6</v>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="84">
@@ -3568,28 +3568,28 @@
         <v>17</v>
       </c>
       <c r="E84" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F84" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G84" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H84" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I84" t="str">
-        <v>3 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="J84" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K84">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L84" t="str">
-        <v/>
+        <v>Thứ 6</v>
       </c>
     </row>
     <row r="85">
@@ -3609,25 +3609,25 @@
         <v>1 tiết</v>
       </c>
       <c r="F85" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G85" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H85" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I85" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J85" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K85">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L85" t="str">
-        <v/>
+        <v>Thứ 3</v>
       </c>
     </row>
   </sheetData>
@@ -3639,7 +3639,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B13"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -3675,7 +3675,7 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Khóa cứng Tiết 5 Thứ 7</v>
+        <v>Khóa cứng Tiết 5 Thứ 7 (Tan sớm)</v>
       </c>
       <c r="B5" t="str">
         <v>ĐẠT 100%</v>
@@ -3691,71 +3691,63 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v/>
+        <v>Cơ cấu tiết các thứ (T2:4, T3:4, T4:5/4, T5:5, T6:5, T7:4) [Cấu hình]</v>
       </c>
       <c r="B7" t="str">
-        <v/>
+        <v>ĐẠT 100%</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>THỐNG KÊ PHÂN BỔ NGÀY NGHỈ</v>
+        <v>Phân bổ số tiết TKB thực tế (K8,9: 27t; K6,7: 26t)</v>
       </c>
       <c r="B8" t="str">
-        <v>SỐ GIÁO VIÊN ĐƯỢC NGHỈ</v>
+        <v>ĐẠT 100%</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Thứ 2</v>
+        <v>Nghỉ Tiết 5 Thứ 2 (Tan trường sau Chào cờ chiều)</v>
       </c>
       <c r="B9" t="str">
-        <v>2 giáo viên</v>
+        <v>ĐẠT 100%</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Thứ 3</v>
+        <v>Vị trí Chào cờ (T1/T4 T2) &amp; SHL (Tiết 4 T7)</v>
       </c>
       <c r="B10" t="str">
-        <v>9 giáo viên</v>
+        <v>ĐẠT 100%</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Thứ 4</v>
+        <v/>
       </c>
       <c r="B11" t="str">
-        <v>14 giáo viên</v>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Thứ 5</v>
+        <v>Tổng giáo viên phân tích</v>
       </c>
       <c r="B12" t="str">
-        <v>8 giáo viên</v>
+        <v>84 giáo viên</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Thứ 6</v>
+        <v>Tổng số tiết đã xếp</v>
       </c>
       <c r="B13" t="str">
-        <v>7 giáo viên</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>Thứ 7</v>
-      </c>
-      <c r="B14" t="str">
-        <v>23 giáo viên</v>
+        <v>917 / 917 tiết (100%)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B13"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix: support Excel day format S.T2-S.T7/C.T2-C.T7, sync 100% official timetable from TKB_L1_2026-2027.xlsx for 84 teachers and 51 classes
</commit_message>
<xml_diff>
--- a/Bao_Cao_Kiem_Dinh_THCS_TKB_FET.xlsx
+++ b/Bao_Cao_Kiem_Dinh_THCS_TKB_FET.xlsx
@@ -452,16 +452,16 @@
         <v>14</v>
       </c>
       <c r="E2" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F2" t="str">
         <v>3 tiết</v>
       </c>
       <c r="G2" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="H2" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I2" t="str">
         <v>4 tiết</v>
@@ -531,13 +531,13 @@
         <v>2 tiết</v>
       </c>
       <c r="F4" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G4" t="str">
         <v>5 tiết</v>
       </c>
       <c r="H4" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I4" t="str">
         <v>4 tiết</v>
@@ -572,13 +572,13 @@
         <v>4 tiết</v>
       </c>
       <c r="G5" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H5" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I5" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J5" t="str">
         <v>NGHỈ</v>
@@ -718,7 +718,7 @@
         <v>16</v>
       </c>
       <c r="E9" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F9" t="str">
         <v>NGHỈ</v>
@@ -730,7 +730,7 @@
         <v>3 tiết</v>
       </c>
       <c r="I9" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J9" t="str">
         <v>4 tiết</v>
@@ -756,28 +756,28 @@
         <v>20</v>
       </c>
       <c r="E10" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="F10" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="G10" t="str">
-        <v>6 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H10" t="str">
         <v>6 tiết</v>
       </c>
       <c r="I10" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J10" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K10">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L10" t="str">
-        <v>Thứ 2, Thứ 7</v>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="11">
@@ -873,16 +873,16 @@
         <v>2 tiết</v>
       </c>
       <c r="F13" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G13" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H13" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I13" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J13" t="str">
         <v>4 tiết</v>
@@ -908,10 +908,10 @@
         <v>17</v>
       </c>
       <c r="E14" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F14" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G14" t="str">
         <v>NGHỈ</v>
@@ -984,13 +984,13 @@
         <v>14</v>
       </c>
       <c r="E16" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F16" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="G16" t="str">
-        <v>2 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H16" t="str">
         <v>2 tiết</v>
@@ -999,7 +999,7 @@
         <v>2 tiết</v>
       </c>
       <c r="J16" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K16">
         <v>1</v>
@@ -1025,16 +1025,16 @@
         <v>2 tiết</v>
       </c>
       <c r="F17" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G17" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H17" t="str">
         <v>3 tiết</v>
       </c>
       <c r="I17" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J17" t="str">
         <v>NGHỈ</v>
@@ -1098,19 +1098,19 @@
         <v>17</v>
       </c>
       <c r="E19" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F19" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G19" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H19" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I19" t="str">
-        <v>7 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J19" t="str">
         <v>NGHỈ</v>
@@ -1212,28 +1212,28 @@
         <v>12</v>
       </c>
       <c r="E22" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="F22" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G22" t="str">
         <v>2 tiết</v>
       </c>
       <c r="H22" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I22" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J22" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L22" t="str">
-        <v>Thứ 2, Thứ 7</v>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="23">
@@ -1288,19 +1288,19 @@
         <v>14</v>
       </c>
       <c r="E24" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F24" t="str">
         <v>2 tiết</v>
       </c>
       <c r="G24" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H24" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="I24" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J24" t="str">
         <v>3 tiết</v>
@@ -1326,7 +1326,7 @@
         <v>17</v>
       </c>
       <c r="E25" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F25" t="str">
         <v>NGHỈ</v>
@@ -1335,7 +1335,7 @@
         <v>7 tiết</v>
       </c>
       <c r="H25" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I25" t="str">
         <v>4 tiết</v>
@@ -1373,10 +1373,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="H26" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I26" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J26" t="str">
         <v>4 tiết</v>
@@ -1402,28 +1402,28 @@
         <v>15</v>
       </c>
       <c r="E27" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F27" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G27" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H27" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I27" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J27" t="str">
         <v>4 tiết</v>
       </c>
       <c r="K27">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L27" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="28">
@@ -1478,19 +1478,19 @@
         <v>16</v>
       </c>
       <c r="E29" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F29" t="str">
-        <v>6 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G29" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H29" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I29" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J29" t="str">
         <v>3 tiết</v>
@@ -1522,13 +1522,13 @@
         <v>NGHỈ</v>
       </c>
       <c r="G30" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="H30" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I30" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J30" t="str">
         <v>2 tiết</v>
@@ -1595,13 +1595,13 @@
         <v>3 tiết</v>
       </c>
       <c r="F32" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G32" t="str">
         <v>4 tiết</v>
       </c>
       <c r="H32" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I32" t="str">
         <v>NGHỈ</v>
@@ -1747,13 +1747,13 @@
         <v>1 tiết</v>
       </c>
       <c r="F36" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="G36" t="str">
         <v>4 tiết</v>
       </c>
       <c r="H36" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I36" t="str">
         <v>NGHỈ</v>
@@ -1858,28 +1858,28 @@
         <v>18</v>
       </c>
       <c r="E39" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F39" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="G39" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H39" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I39" t="str">
         <v>2 tiết</v>
       </c>
       <c r="J39" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="K39">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L39" t="str">
-        <v/>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="40">
@@ -1902,13 +1902,13 @@
         <v>1 tiết</v>
       </c>
       <c r="G40" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="H40" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I40" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J40" t="str">
         <v>4 tiết</v>
@@ -1934,19 +1934,19 @@
         <v>16</v>
       </c>
       <c r="E41" t="str">
-        <v>1 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="F41" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G41" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H41" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I41" t="str">
-        <v>5 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J41" t="str">
         <v>4 tiết</v>
@@ -2124,28 +2124,28 @@
         <v>21</v>
       </c>
       <c r="E46" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F46" t="str">
         <v>4 tiết</v>
       </c>
       <c r="G46" t="str">
-        <v>2 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H46" t="str">
         <v>6 tiết</v>
       </c>
       <c r="I46" t="str">
-        <v>6 tiết</v>
+        <v>7 tiết</v>
       </c>
       <c r="J46" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="K46">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L46" t="str">
-        <v/>
+        <v>Thứ 4, Thứ 7</v>
       </c>
     </row>
     <row r="47">
@@ -2162,7 +2162,7 @@
         <v>13</v>
       </c>
       <c r="E47" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="F47" t="str">
         <v>NGHỈ</v>
@@ -2174,7 +2174,7 @@
         <v>1 tiết</v>
       </c>
       <c r="I47" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J47" t="str">
         <v>3 tiết</v>
@@ -2206,16 +2206,16 @@
         <v>4 tiết</v>
       </c>
       <c r="G48" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H48" t="str">
-        <v>3 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="I48" t="str">
         <v>2 tiết</v>
       </c>
       <c r="J48" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K48">
         <v>0</v>
@@ -2244,13 +2244,13 @@
         <v>2 tiết</v>
       </c>
       <c r="G49" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="H49" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="I49" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J49" t="str">
         <v>5 tiết</v>
@@ -2282,13 +2282,13 @@
         <v>2 tiết</v>
       </c>
       <c r="G50" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H50" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="I50" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J50" t="str">
         <v>3 tiết</v>
@@ -2314,22 +2314,22 @@
         <v>16</v>
       </c>
       <c r="E51" t="str">
-        <v>2 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="F51" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G51" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="H51" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I51" t="str">
-        <v>5 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J51" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="K51">
         <v>1</v>
@@ -2393,16 +2393,16 @@
         <v>2 tiết</v>
       </c>
       <c r="F53" t="str">
+        <v>4 tiết</v>
+      </c>
+      <c r="G53" t="str">
+        <v>4 tiết</v>
+      </c>
+      <c r="H53" t="str">
+        <v>4 tiết</v>
+      </c>
+      <c r="I53" t="str">
         <v>5 tiết</v>
-      </c>
-      <c r="G53" t="str">
-        <v>4 tiết</v>
-      </c>
-      <c r="H53" t="str">
-        <v>4 tiết</v>
-      </c>
-      <c r="I53" t="str">
-        <v>4 tiết</v>
       </c>
       <c r="J53" t="str">
         <v>NGHỈ</v>
@@ -2466,28 +2466,28 @@
         <v>16</v>
       </c>
       <c r="E55" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F55" t="str">
         <v>1 tiết</v>
       </c>
       <c r="G55" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="H55" t="str">
+        <v>4 tiết</v>
+      </c>
+      <c r="I55" t="str">
+        <v>3 tiết</v>
+      </c>
+      <c r="J55" t="str">
         <v>5 tiết</v>
       </c>
-      <c r="I55" t="str">
-        <v>4 tiết</v>
-      </c>
-      <c r="J55" t="str">
-        <v>3 tiết</v>
-      </c>
       <c r="K55">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L55" t="str">
-        <v>Thứ 4</v>
+        <v/>
       </c>
     </row>
     <row r="56">
@@ -2656,19 +2656,19 @@
         <v>14</v>
       </c>
       <c r="E60" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F60" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="G60" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H60" t="str">
-        <v>5 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="I60" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J60" t="str">
         <v>4 tiết</v>
@@ -2706,10 +2706,10 @@
         <v>3 tiết</v>
       </c>
       <c r="I61" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J61" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K61">
         <v>1</v>
@@ -2732,28 +2732,28 @@
         <v>18</v>
       </c>
       <c r="E62" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="F62" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G62" t="str">
-        <v>6 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H62" t="str">
-        <v>6 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="I62" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J62" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="K62">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L62" t="str">
-        <v>Thứ 2, Thứ 7</v>
+        <v>Thứ 7</v>
       </c>
     </row>
     <row r="63">
@@ -2770,22 +2770,22 @@
         <v>15</v>
       </c>
       <c r="E63" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="F63" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G63" t="str">
         <v>3 tiết</v>
       </c>
       <c r="H63" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="I63" t="str">
         <v>NGHỈ</v>
       </c>
       <c r="J63" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="K63">
         <v>1</v>
@@ -2887,25 +2887,25 @@
         <v>2 tiết</v>
       </c>
       <c r="F66" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G66" t="str">
         <v>2 tiết</v>
       </c>
       <c r="H66" t="str">
-        <v>4 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="I66" t="str">
-        <v>1 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="J66" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L66" t="str">
-        <v/>
+        <v>Thứ 5</v>
       </c>
     </row>
     <row r="67">
@@ -2922,13 +2922,13 @@
         <v>16</v>
       </c>
       <c r="E67" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F67" t="str">
         <v>4 tiết</v>
       </c>
       <c r="G67" t="str">
-        <v>1 tiết</v>
+        <v>NGHỈ</v>
       </c>
       <c r="H67" t="str">
         <v>4 tiết</v>
@@ -2940,10 +2940,10 @@
         <v>3 tiết</v>
       </c>
       <c r="K67">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L67" t="str">
-        <v/>
+        <v>Thứ 4</v>
       </c>
     </row>
     <row r="68">
@@ -3007,10 +3007,10 @@
         <v>NGHỈ</v>
       </c>
       <c r="H69" t="str">
-        <v>3 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I69" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J69" t="str">
         <v>3 tiết</v>
@@ -3083,13 +3083,13 @@
         <v>3 tiết</v>
       </c>
       <c r="H71" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I71" t="str">
-        <v>4 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="J71" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="K71">
         <v>0</v>
@@ -3156,22 +3156,22 @@
         <v>NGHỈ</v>
       </c>
       <c r="G73" t="str">
-        <v>2 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="H73" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="I73" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J73" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="K73">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L73" t="str">
-        <v>Thứ 3, Thứ 5</v>
+        <v>Thứ 3</v>
       </c>
     </row>
     <row r="74">
@@ -3229,16 +3229,16 @@
         <v>3 tiết</v>
       </c>
       <c r="F75" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G75" t="str">
-        <v>5 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="H75" t="str">
-        <v>1 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="I75" t="str">
-        <v>3 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="J75" t="str">
         <v>NGHỈ</v>
@@ -3267,16 +3267,16 @@
         <v>2 tiết</v>
       </c>
       <c r="F76" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="G76" t="str">
-        <v>4 tiết</v>
+        <v>6 tiết</v>
       </c>
       <c r="H76" t="str">
-        <v>3 tiết</v>
+        <v>5 tiết</v>
       </c>
       <c r="I76" t="str">
-        <v>5 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="J76" t="str">
         <v>NGHỈ</v>
@@ -3340,10 +3340,10 @@
         <v>12</v>
       </c>
       <c r="E78" t="str">
-        <v>1 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="F78" t="str">
-        <v>2 tiết</v>
+        <v>1 tiết</v>
       </c>
       <c r="G78" t="str">
         <v>3 tiết</v>
@@ -3533,25 +3533,25 @@
         <v>1 tiết</v>
       </c>
       <c r="F83" t="str">
-        <v>2 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="G83" t="str">
-        <v>NGHỈ</v>
+        <v>2 tiết</v>
       </c>
       <c r="H83" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="I83" t="str">
-        <v>4 tiết</v>
+        <v>2 tiết</v>
       </c>
       <c r="J83" t="str">
         <v>3 tiết</v>
       </c>
       <c r="K83">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L83" t="str">
-        <v>Thứ 4</v>
+        <v/>
       </c>
     </row>
     <row r="84">
@@ -3571,10 +3571,10 @@
         <v>2 tiết</v>
       </c>
       <c r="F84" t="str">
-        <v>4 tiết</v>
+        <v>3 tiết</v>
       </c>
       <c r="G84" t="str">
-        <v>3 tiết</v>
+        <v>4 tiết</v>
       </c>
       <c r="H84" t="str">
         <v>4 tiết</v>

</xml_diff>